<commit_message>
Adding stella lr trainings
</commit_message>
<xml_diff>
--- a/Embedding Performances.xlsx
+++ b/Embedding Performances.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\Kevin\Projects\trend-analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8553BFB-97A2-42EE-9E46-AE295480C60A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE2C19C4-2676-4E8B-B1C7-B9B4058EB375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6105" yWindow="2010" windowWidth="21600" windowHeight="11295" xr2:uid="{D74B7566-5B2D-48D0-8971-D6203F1B9797}"/>
+    <workbookView xWindow="-17655" yWindow="2205" windowWidth="17010" windowHeight="10290" xr2:uid="{D74B7566-5B2D-48D0-8971-D6203F1B9797}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
   <si>
     <t>Simulated data</t>
   </si>
@@ -122,13 +122,16 @@
     <t>0.9763/0.9787</t>
   </si>
   <si>
-    <t>0.9839/0.9852</t>
-  </si>
-  <si>
-    <t>0.9626/0.9677</t>
-  </si>
-  <si>
-    <t>0.9750/0.9777</t>
+    <t>LR (AUROC/AUPR)</t>
+  </si>
+  <si>
+    <t>0.9830/0.9843</t>
+  </si>
+  <si>
+    <t>0.9634/0.9683</t>
+  </si>
+  <si>
+    <t>0.9745/0.9772</t>
   </si>
 </sst>
 </file>
@@ -184,9 +187,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -224,7 +227,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -330,7 +333,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -472,7 +475,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -509,7 +512,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -550,7 +553,7 @@
         <v>21</v>
       </c>
       <c r="G3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H3" t="s">
         <v>25</v>
@@ -576,7 +579,7 @@
         <v>22</v>
       </c>
       <c r="G4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H4" t="s">
         <v>27</v>
@@ -602,7 +605,7 @@
         <v>23</v>
       </c>
       <c r="G5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H5" t="s">
         <v>26</v>

</xml_diff>